<commit_message>
feat: add new xlsx header - line
</commit_message>
<xml_diff>
--- a/src/main/resources/qm/public/resources/qSHProductImportSchema_vi.xlsx
+++ b/src/main/resources/qm/public/resources/qSHProductImportSchema_vi.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Qcadoo_demo_clone\mes\mes-plugins\fti-plugins-qm\src\main\resources\qm\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35CA6CA7-25A3-4C63-962E-348065A0E0C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5DA73FF-F676-467E-83D3-13F1CFC7BC0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1C3DD0E6-ED60-435A-92B4-4D6BBCAE0B6F}"/>
+    <workbookView xWindow="5235" yWindow="3405" windowWidth="21600" windowHeight="11235" xr2:uid="{1C3DD0E6-ED60-435A-92B4-4D6BBCAE0B6F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>